<commit_message>
feat: harden universal estimate generation
</commit_message>
<xml_diff>
--- a/Универсальный_расчет_стоимости_MONSters_v2_шаблон_для_разработчиков.xlsx
+++ b/Универсальный_расчет_стоимости_MONSters_v2_шаблон_для_разработчиков.xlsx
@@ -18644,7 +18644,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
@@ -18712,8 +18712,7 @@
         <v>389</v>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF('Справочник типов'!$A$2:$A$27,Ввод!$B$5)</f>
-        <v>0</v>
+        <f>IF(ISNUMBER(MATCH('Ввод'!$B$5,'Справочник типов'!$A$2:$A$27,0)),1,0)</f>
       </c>
       <c r="C6" s="5" t="s">
         <v>390</v>

</xml_diff>